<commit_message>
Bitacoras 9 y 10
</commit_message>
<xml_diff>
--- a/Bitacora_9.xlsx
+++ b/Bitacora_9.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29825"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://btgpactual-my.sharepoint.com/personal/juan_alcala_btgpactual_com/Documents/Escritorio/Bitacoras/bitacoras/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://btgpactual-my.sharepoint.com/personal/juan_alcala_btgpactual_com/Documents/Bitacoras/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="393" documentId="8_{B11B8281-ACE1-4350-8618-021BE984FAB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{426A4383-DE27-40D1-B862-0B8F07EEB799}"/>
+  <xr:revisionPtr revIDLastSave="399" documentId="8_{B11B8281-ACE1-4350-8618-021BE984FAB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2A1DE24-DB0F-4A6B-A0D0-C7130A89F612}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-18615" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="5" r:id="rId1"/>
@@ -508,6 +508,9 @@
     <t>BTG Pactual</t>
   </si>
   <si>
+    <t xml:space="preserve">Desde 01/02/2026  hasta 15/02/2025 </t>
+  </si>
+  <si>
     <t xml:space="preserve">Santiago Pulgarin Vazquez </t>
   </si>
   <si>
@@ -673,6 +676,51 @@
     <t xml:space="preserve">Y/O COMENTARIOS  REALIZADOS POR LAS PERSONAS CON ROL DE: APRENDIZ Y/O JEFE INMEDIATO </t>
   </si>
   <si>
+    <t>Modifiqué la consulta de portafolio para que aparecieran los datos de la cuenta omnibus</t>
+  </si>
+  <si>
+    <t>Los cambios fueron integrados y subidos al repositorio en Azure</t>
+  </si>
+  <si>
+    <t>No se presentaron dificultades</t>
+  </si>
+  <si>
+    <t>Resolví los code smells identificados</t>
+  </si>
+  <si>
+    <t>SonarQube confirmó la resolución y los ajustes quedaron registrados en Azure</t>
+  </si>
+  <si>
+    <t>Mejoré la calidad del código</t>
+  </si>
+  <si>
+    <t>Realicé un curso de AWS y otros temas en mis tiempos libres</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> materiales de estudio completados en AWS</t>
+  </si>
+  <si>
+    <t>Actividad de formación personal</t>
+  </si>
+  <si>
+    <t>Estuve probando ocasionalmente funcionalidades en Dominus Dev</t>
+  </si>
+  <si>
+    <t>Pruebas realizadas y registradas en entornos de desarrollo</t>
+  </si>
+  <si>
+    <t>Actividad exploratoria sin incidencias</t>
+  </si>
+  <si>
+    <t>Apoyé ocasionalmente a compañeros en sus tareas</t>
+  </si>
+  <si>
+    <t>Colaboraciones registradas en repositorio y comunicación interna</t>
+  </si>
+  <si>
+    <t>Apoyo puntual, sin dificultades</t>
+  </si>
+  <si>
     <t xml:space="preserve">Decreto 055 de 2015, por el cual se reglamenta la afiliación de estudiantes al Sistema General de Riesgos Laborales y se dictan otras disposiciones </t>
   </si>
   <si>
@@ -844,60 +892,12 @@
   <si>
     <t>firma el instructor que recibe la bitácora</t>
   </si>
-  <si>
-    <t xml:space="preserve">Desde 01/02/2026  hasta 15/02/2025 </t>
-  </si>
-  <si>
-    <t>Modifiqué la consulta de portafolio para que aparecieran los datos de la cuenta omnibus</t>
-  </si>
-  <si>
-    <t>Resolví los code smells identificados</t>
-  </si>
-  <si>
-    <t>Realicé un curso de AWS y otros temas en mis tiempos libres</t>
-  </si>
-  <si>
-    <t>Estuve probando ocasionalmente funcionalidades en Dominus Dev</t>
-  </si>
-  <si>
-    <t>Apoyé ocasionalmente a compañeros en sus tareas</t>
-  </si>
-  <si>
-    <t>Los cambios fueron integrados y subidos al repositorio en Azure</t>
-  </si>
-  <si>
-    <t>SonarQube confirmó la resolución y los ajustes quedaron registrados en Azure</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> materiales de estudio completados en AWS</t>
-  </si>
-  <si>
-    <t>Pruebas realizadas y registradas en entornos de desarrollo</t>
-  </si>
-  <si>
-    <t>Colaboraciones registradas en repositorio y comunicación interna</t>
-  </si>
-  <si>
-    <t>No se presentaron dificultades</t>
-  </si>
-  <si>
-    <t>Mejoré la calidad del código</t>
-  </si>
-  <si>
-    <t>Actividad de formación personal</t>
-  </si>
-  <si>
-    <t>Actividad exploratoria sin incidencias</t>
-  </si>
-  <si>
-    <t>Apoyo puntual, sin dificultades</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="39" x14ac:knownFonts="1">
+  <fonts count="39">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3771,22 +3771,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1132417</xdr:colOff>
+      <xdr:colOff>1304925</xdr:colOff>
       <xdr:row>74</xdr:row>
-      <xdr:rowOff>42333</xdr:rowOff>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>1471364</xdr:colOff>
+      <xdr:colOff>828675</xdr:colOff>
       <xdr:row>76</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Imagen 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E37CF4F-5E0A-479F-99C4-6E346AA80547}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EFBAC735-FEBB-CC79-1066-F3E82B92B268}"/>
             </a:ext>
             <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
               <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{9F75D9DB-16BF-493F-916C-CBC4DAF8756A}"/>
@@ -3805,8 +3805,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10001250" y="23759583"/>
-          <a:ext cx="2519114" cy="519642"/>
+          <a:off x="10182225" y="23726775"/>
+          <a:ext cx="1704975" cy="438150"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4185,7 +4185,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:H59"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.42578125" customWidth="1"/>
     <col min="2" max="2" width="47.42578125" style="58" customWidth="1"/>
@@ -4195,7 +4195,7 @@
     <col min="7" max="7" width="46.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:8" ht="28.5" customHeight="1">
       <c r="B1" s="67"/>
       <c r="C1" s="68"/>
       <c r="D1" s="68"/>
@@ -4206,7 +4206,7 @@
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
     </row>
-    <row r="2" spans="2:8" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8" ht="28.5" customHeight="1">
       <c r="B2" s="70"/>
       <c r="C2" s="54"/>
       <c r="D2" s="54"/>
@@ -4217,7 +4217,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
     </row>
-    <row r="3" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:8" ht="25.5" customHeight="1">
       <c r="B3" s="172" t="s">
         <v>2</v>
       </c>
@@ -4228,7 +4228,7 @@
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
     </row>
-    <row r="4" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" ht="25.5" customHeight="1">
       <c r="B4" s="175" t="s">
         <v>3</v>
       </c>
@@ -4239,7 +4239,7 @@
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
     </row>
-    <row r="5" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" ht="25.5" customHeight="1">
       <c r="B5" s="178" t="s">
         <v>4</v>
       </c>
@@ -4250,7 +4250,7 @@
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
     </row>
-    <row r="6" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8" ht="25.5" customHeight="1">
       <c r="B6" s="175" t="s">
         <v>5</v>
       </c>
@@ -4261,7 +4261,7 @@
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
     </row>
-    <row r="7" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" ht="25.5" customHeight="1">
       <c r="B7" s="172" t="s">
         <v>6</v>
       </c>
@@ -4272,7 +4272,7 @@
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
     </row>
-    <row r="8" spans="2:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8" ht="31.5" customHeight="1">
       <c r="B8" s="72" t="s">
         <v>7</v>
       </c>
@@ -4285,7 +4285,7 @@
       <c r="E8" s="182"/>
       <c r="H8" s="7"/>
     </row>
-    <row r="9" spans="2:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" ht="25.5" customHeight="1">
       <c r="B9" s="183" t="s">
         <v>10</v>
       </c>
@@ -4295,7 +4295,7 @@
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
     </row>
-    <row r="10" spans="2:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8" ht="17.25" customHeight="1">
       <c r="B10" s="186" t="s">
         <v>11</v>
       </c>
@@ -4303,7 +4303,7 @@
       <c r="D10" s="187"/>
       <c r="E10" s="188"/>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8">
       <c r="B11" s="189" t="s">
         <v>12</v>
       </c>
@@ -4311,7 +4311,7 @@
       <c r="D11" s="190"/>
       <c r="E11" s="191"/>
     </row>
-    <row r="12" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:8" ht="51" customHeight="1">
       <c r="B12" s="168" t="s">
         <v>13</v>
       </c>
@@ -4321,13 +4321,13 @@
       <c r="F12" s="1"/>
       <c r="G12" s="36"/>
     </row>
-    <row r="13" spans="2:8" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" ht="12.75" customHeight="1">
       <c r="B13" s="78"/>
       <c r="C13" s="79"/>
       <c r="D13" s="79"/>
       <c r="E13" s="80"/>
     </row>
-    <row r="14" spans="2:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" ht="27.75" customHeight="1">
       <c r="B14" s="201" t="s">
         <v>14</v>
       </c>
@@ -4335,7 +4335,7 @@
       <c r="D14" s="202"/>
       <c r="E14" s="203"/>
     </row>
-    <row r="15" spans="2:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:8" ht="21.75" customHeight="1">
       <c r="B15" s="204" t="s">
         <v>15</v>
       </c>
@@ -4343,7 +4343,7 @@
       <c r="D15" s="205"/>
       <c r="E15" s="206"/>
     </row>
-    <row r="16" spans="2:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:8" ht="21.75" customHeight="1">
       <c r="B16" s="204" t="s">
         <v>16</v>
       </c>
@@ -4351,7 +4351,7 @@
       <c r="D16" s="205"/>
       <c r="E16" s="206"/>
     </row>
-    <row r="17" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" ht="30" customHeight="1">
       <c r="B17" s="210" t="s">
         <v>17</v>
       </c>
@@ -4359,7 +4359,7 @@
       <c r="D17" s="211"/>
       <c r="E17" s="212"/>
     </row>
-    <row r="18" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" ht="21.75" customHeight="1">
       <c r="B18" s="204" t="s">
         <v>18</v>
       </c>
@@ -4367,7 +4367,7 @@
       <c r="D18" s="205"/>
       <c r="E18" s="206"/>
     </row>
-    <row r="19" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" ht="21.75" customHeight="1">
       <c r="B19" s="204" t="s">
         <v>19</v>
       </c>
@@ -4375,7 +4375,7 @@
       <c r="D19" s="205"/>
       <c r="E19" s="206"/>
     </row>
-    <row r="20" spans="2:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" ht="21.75" customHeight="1">
       <c r="B20" s="207" t="s">
         <v>20</v>
       </c>
@@ -4383,7 +4383,7 @@
       <c r="D20" s="208"/>
       <c r="E20" s="209"/>
     </row>
-    <row r="21" spans="2:6" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" ht="27" customHeight="1">
       <c r="B21" s="168" t="s">
         <v>21</v>
       </c>
@@ -4391,7 +4391,7 @@
       <c r="D21" s="170"/>
       <c r="E21" s="171"/>
     </row>
-    <row r="22" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" ht="15" customHeight="1">
       <c r="B22" s="189" t="s">
         <v>22</v>
       </c>
@@ -4401,13 +4401,13 @@
       </c>
       <c r="E22" s="191"/>
     </row>
-    <row r="23" spans="2:6" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" ht="5.25" customHeight="1">
       <c r="B23" s="192"/>
       <c r="C23" s="193"/>
       <c r="D23" s="193"/>
       <c r="E23" s="194"/>
     </row>
-    <row r="24" spans="2:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" ht="14.25" customHeight="1">
       <c r="B24" s="73" t="s">
         <v>23</v>
       </c>
@@ -4420,7 +4420,7 @@
       <c r="E24" s="196"/>
       <c r="F24" s="8"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6">
       <c r="B25" s="74" t="s">
         <v>26</v>
       </c>
@@ -4430,7 +4430,7 @@
       <c r="D25" s="197"/>
       <c r="E25" s="198"/>
     </row>
-    <row r="26" spans="2:6" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" ht="31.5">
       <c r="B26" s="62" t="s">
         <v>28</v>
       </c>
@@ -4440,7 +4440,7 @@
       <c r="D26" s="197"/>
       <c r="E26" s="198"/>
     </row>
-    <row r="27" spans="2:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" ht="45">
       <c r="B27" s="64" t="s">
         <v>30</v>
       </c>
@@ -4450,7 +4450,7 @@
       <c r="D27" s="197"/>
       <c r="E27" s="198"/>
     </row>
-    <row r="28" spans="2:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" ht="21" customHeight="1">
       <c r="B28" s="74" t="s">
         <v>32</v>
       </c>
@@ -4460,7 +4460,7 @@
       <c r="D28" s="197"/>
       <c r="E28" s="198"/>
     </row>
-    <row r="29" spans="2:6" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" ht="44.25" customHeight="1">
       <c r="B29" s="74" t="s">
         <v>34</v>
       </c>
@@ -4474,7 +4474,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="2:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" ht="36.75" customHeight="1">
       <c r="B30" s="74" t="s">
         <v>37</v>
       </c>
@@ -4488,7 +4488,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="2:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" ht="30">
       <c r="B31" s="74" t="s">
         <v>40</v>
       </c>
@@ -4498,7 +4498,7 @@
       <c r="D31" s="197"/>
       <c r="E31" s="198"/>
     </row>
-    <row r="32" spans="2:6" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" ht="65.25" customHeight="1">
       <c r="B32" s="74" t="s">
         <v>42</v>
       </c>
@@ -4512,7 +4512,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="2:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:5" ht="75">
       <c r="B33" s="74" t="s">
         <v>45</v>
       </c>
@@ -4522,7 +4522,7 @@
       <c r="D33" s="197"/>
       <c r="E33" s="198"/>
     </row>
-    <row r="34" spans="2:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:5" ht="60">
       <c r="B34" s="74" t="s">
         <v>47</v>
       </c>
@@ -4532,7 +4532,7 @@
       <c r="D34" s="197"/>
       <c r="E34" s="198"/>
     </row>
-    <row r="35" spans="2:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:5" ht="60">
       <c r="B35" s="74" t="s">
         <v>49</v>
       </c>
@@ -4542,7 +4542,7 @@
       <c r="D35" s="197"/>
       <c r="E35" s="198"/>
     </row>
-    <row r="36" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:5" ht="45">
       <c r="B36" s="74" t="s">
         <v>51</v>
       </c>
@@ -4552,7 +4552,7 @@
       <c r="D36" s="197"/>
       <c r="E36" s="198"/>
     </row>
-    <row r="37" spans="2:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:5" ht="60">
       <c r="B37" s="74" t="s">
         <v>53</v>
       </c>
@@ -4562,7 +4562,7 @@
       <c r="D37" s="197"/>
       <c r="E37" s="198"/>
     </row>
-    <row r="38" spans="2:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:5" ht="60">
       <c r="B38" s="74" t="s">
         <v>55</v>
       </c>
@@ -4572,7 +4572,7 @@
       <c r="D38" s="197"/>
       <c r="E38" s="198"/>
     </row>
-    <row r="39" spans="2:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:5" ht="60">
       <c r="B39" s="74" t="s">
         <v>32</v>
       </c>
@@ -4582,7 +4582,7 @@
       <c r="D39" s="197"/>
       <c r="E39" s="198"/>
     </row>
-    <row r="40" spans="2:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:5" ht="60">
       <c r="B40" s="74" t="s">
         <v>58</v>
       </c>
@@ -4592,7 +4592,7 @@
       <c r="D40" s="197"/>
       <c r="E40" s="198"/>
     </row>
-    <row r="41" spans="2:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:5" ht="60">
       <c r="B41" s="74" t="s">
         <v>60</v>
       </c>
@@ -4602,7 +4602,7 @@
       <c r="D41" s="197"/>
       <c r="E41" s="198"/>
     </row>
-    <row r="42" spans="2:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:5" ht="60">
       <c r="B42" s="74" t="s">
         <v>58</v>
       </c>
@@ -4612,7 +4612,7 @@
       <c r="D42" s="197"/>
       <c r="E42" s="198"/>
     </row>
-    <row r="43" spans="2:5" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:5" ht="409.5">
       <c r="B43" s="74" t="s">
         <v>63</v>
       </c>
@@ -4626,7 +4626,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:5" ht="30">
       <c r="B44" s="74" t="s">
         <v>66</v>
       </c>
@@ -4636,7 +4636,7 @@
       <c r="D44" s="197"/>
       <c r="E44" s="198"/>
     </row>
-    <row r="45" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:5" ht="30">
       <c r="B45" s="74" t="s">
         <v>68</v>
       </c>
@@ -4646,7 +4646,7 @@
       <c r="D45" s="197"/>
       <c r="E45" s="198"/>
     </row>
-    <row r="46" spans="2:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:5" ht="30">
       <c r="B46" s="74" t="s">
         <v>70</v>
       </c>
@@ -4656,7 +4656,7 @@
       <c r="D46" s="197"/>
       <c r="E46" s="198"/>
     </row>
-    <row r="47" spans="2:5" ht="127.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:5" ht="127.5" customHeight="1">
       <c r="B47" s="74" t="s">
         <v>72</v>
       </c>
@@ -4670,7 +4670,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:5" ht="45">
       <c r="B48" s="74" t="s">
         <v>75</v>
       </c>
@@ -4680,7 +4680,7 @@
       <c r="D48" s="197"/>
       <c r="E48" s="198"/>
     </row>
-    <row r="49" spans="2:5" ht="146.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:5" ht="146.25" customHeight="1">
       <c r="B49" s="74" t="s">
         <v>77</v>
       </c>
@@ -4694,7 +4694,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="50" spans="2:5" ht="339.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:5" ht="339.75" customHeight="1">
       <c r="B50" s="74" t="s">
         <v>80</v>
       </c>
@@ -4708,7 +4708,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="51" spans="2:5" ht="84.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:5" ht="84.75" customHeight="1">
       <c r="B51" s="74" t="s">
         <v>84</v>
       </c>
@@ -4722,7 +4722,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="52" spans="2:5" ht="90" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:5" ht="90">
       <c r="B52" s="74" t="s">
         <v>87</v>
       </c>
@@ -4732,7 +4732,7 @@
       <c r="D52" s="197"/>
       <c r="E52" s="198"/>
     </row>
-    <row r="53" spans="2:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:5" ht="75">
       <c r="B53" s="74" t="s">
         <v>89</v>
       </c>
@@ -4742,7 +4742,7 @@
       <c r="D53" s="197"/>
       <c r="E53" s="198"/>
     </row>
-    <row r="54" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:5" ht="45">
       <c r="B54" s="74" t="s">
         <v>91</v>
       </c>
@@ -4752,7 +4752,7 @@
       <c r="D54" s="197"/>
       <c r="E54" s="198"/>
     </row>
-    <row r="55" spans="2:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:5" ht="75">
       <c r="B55" s="74" t="s">
         <v>93</v>
       </c>
@@ -4762,7 +4762,7 @@
       <c r="D55" s="197"/>
       <c r="E55" s="198"/>
     </row>
-    <row r="56" spans="2:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:5" ht="75">
       <c r="B56" s="75" t="s">
         <v>95</v>
       </c>
@@ -4772,7 +4772,7 @@
       <c r="D56" s="197"/>
       <c r="E56" s="198"/>
     </row>
-    <row r="57" spans="2:5" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:5" ht="37.5" customHeight="1" thickBot="1">
       <c r="B57" s="76" t="s">
         <v>96</v>
       </c>
@@ -4786,13 +4786,13 @@
         <v>98</v>
       </c>
     </row>
-    <row r="58" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:5">
       <c r="B58" s="55"/>
       <c r="C58" s="55"/>
       <c r="D58" s="56"/>
       <c r="E58" s="56"/>
     </row>
-    <row r="59" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:5">
       <c r="B59" s="57"/>
       <c r="C59" s="57"/>
       <c r="D59" s="56"/>
@@ -4867,7 +4867,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E74A078B-FDD5-4F89-B4CB-7471575D0D0F}">
   <dimension ref="B1:Z84"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2.28515625" style="9" customWidth="1"/>
     <col min="2" max="7" width="32.7109375" style="11" customWidth="1"/>
@@ -4887,7 +4887,7 @@
     <col min="27" max="16384" width="11.42578125" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:26" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:26" ht="29.25" customHeight="1">
       <c r="B1" s="125"/>
       <c r="C1" s="152"/>
       <c r="D1" s="152"/>
@@ -4916,7 +4916,7 @@
       <c r="Y1" s="9"/>
       <c r="Z1" s="9"/>
     </row>
-    <row r="2" spans="2:26" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:26" ht="29.25" customHeight="1">
       <c r="B2" s="154"/>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -4945,7 +4945,7 @@
       <c r="Y2" s="9"/>
       <c r="Z2" s="9"/>
     </row>
-    <row r="3" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:26" ht="24" customHeight="1">
       <c r="B3" s="172" t="s">
         <v>2</v>
       </c>
@@ -4974,7 +4974,7 @@
       <c r="Y3" s="9"/>
       <c r="Z3" s="9"/>
     </row>
-    <row r="4" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:26" ht="24" customHeight="1">
       <c r="B4" s="175" t="s">
         <v>3</v>
       </c>
@@ -5003,7 +5003,7 @@
       <c r="Y4" s="9"/>
       <c r="Z4" s="9"/>
     </row>
-    <row r="5" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:26" ht="24" customHeight="1">
       <c r="B5" s="172" t="s">
         <v>99</v>
       </c>
@@ -5032,7 +5032,7 @@
       <c r="Y5" s="9"/>
       <c r="Z5" s="9"/>
     </row>
-    <row r="6" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:26" ht="24" customHeight="1">
       <c r="B6" s="175" t="s">
         <v>5</v>
       </c>
@@ -5061,7 +5061,7 @@
       <c r="Y6" s="9"/>
       <c r="Z6" s="9"/>
     </row>
-    <row r="7" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:26" ht="24" customHeight="1">
       <c r="B7" s="172" t="s">
         <v>6</v>
       </c>
@@ -5090,7 +5090,7 @@
       <c r="Y7" s="9"/>
       <c r="Z7" s="9"/>
     </row>
-    <row r="8" spans="2:26" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:26" ht="36.75" customHeight="1" thickBot="1">
       <c r="B8" s="156" t="s">
         <v>7</v>
       </c>
@@ -5123,7 +5123,7 @@
       <c r="Y8" s="9"/>
       <c r="Z8" s="9"/>
     </row>
-    <row r="9" spans="2:26" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:26" ht="9" customHeight="1" thickBot="1">
       <c r="B9" s="18"/>
       <c r="C9" s="20"/>
       <c r="D9" s="20"/>
@@ -5150,7 +5150,7 @@
       <c r="Y9" s="9"/>
       <c r="Z9" s="9"/>
     </row>
-    <row r="10" spans="2:26" s="11" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:26" s="11" customFormat="1" ht="29.25" customHeight="1">
       <c r="B10" s="125" t="s">
         <v>100</v>
       </c>
@@ -5170,7 +5170,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:26" ht="18" customHeight="1" thickBot="1">
       <c r="B11" s="120" t="s">
         <v>102</v>
       </c>
@@ -5209,7 +5209,7 @@
       <c r="Y11" s="9"/>
       <c r="Z11" s="9"/>
     </row>
-    <row r="12" spans="2:26" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:26" ht="9" customHeight="1" thickBot="1">
       <c r="B12" s="20"/>
       <c r="D12" s="20"/>
       <c r="E12" s="18"/>
@@ -5235,7 +5235,7 @@
       <c r="Y12" s="9"/>
       <c r="Z12" s="9"/>
     </row>
-    <row r="13" spans="2:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:26" ht="18" customHeight="1">
       <c r="B13" s="135" t="s">
         <v>106</v>
       </c>
@@ -5264,7 +5264,7 @@
       <c r="X13" s="18"/>
       <c r="Y13" s="18"/>
     </row>
-    <row r="14" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:26" ht="18" customHeight="1" thickBot="1">
       <c r="B14" s="231">
         <v>2901692</v>
       </c>
@@ -5293,7 +5293,7 @@
       <c r="X14" s="20"/>
       <c r="Y14" s="20"/>
     </row>
-    <row r="15" spans="2:26" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:26" ht="9.75" customHeight="1" thickBot="1">
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
       <c r="D15" s="15"/>
@@ -5319,7 +5319,7 @@
       <c r="X15" s="15"/>
       <c r="Y15" s="15"/>
     </row>
-    <row r="16" spans="2:26" s="11" customFormat="1" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:26" s="11" customFormat="1" ht="50.25" customHeight="1">
       <c r="B16" s="125" t="s">
         <v>108</v>
       </c>
@@ -5345,7 +5345,7 @@
       <c r="Y16" s="18"/>
       <c r="Z16" s="12"/>
     </row>
-    <row r="17" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:26" ht="18" customHeight="1" thickBot="1">
       <c r="B17" s="231" t="s">
         <v>110</v>
       </c>
@@ -5357,7 +5357,7 @@
         <v>9</v>
       </c>
       <c r="F17" s="236" t="s">
-        <v>202</v>
+        <v>111</v>
       </c>
       <c r="G17" s="237"/>
       <c r="H17" s="20"/>
@@ -5370,7 +5370,7 @@
       <c r="X17" s="20"/>
       <c r="Y17" s="20"/>
     </row>
-    <row r="18" spans="2:26" ht="9.9499999999999993" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:26" ht="9.9499999999999993" customHeight="1" thickBot="1">
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
@@ -5396,7 +5396,7 @@
       <c r="X18" s="15"/>
       <c r="Y18" s="15"/>
     </row>
-    <row r="19" spans="2:26" s="11" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:26" s="11" customFormat="1" ht="45">
       <c r="B19" s="125" t="s">
         <v>53</v>
       </c>
@@ -5426,19 +5426,19 @@
       <c r="Y19" s="18"/>
       <c r="Z19" s="12"/>
     </row>
-    <row r="20" spans="2:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:26" ht="18" customHeight="1">
       <c r="B20" s="231" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C20" s="233"/>
       <c r="D20" s="166" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E20" s="129">
         <v>3104546105</v>
       </c>
       <c r="F20" s="238" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G20" s="239"/>
       <c r="H20" s="20"/>
@@ -5455,7 +5455,7 @@
       <c r="X20" s="20"/>
       <c r="Y20" s="20"/>
     </row>
-    <row r="21" spans="2:26" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:26" ht="8.25" customHeight="1" thickBot="1">
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
       <c r="D21" s="15"/>
@@ -5481,9 +5481,9 @@
       <c r="X21" s="15"/>
       <c r="Y21" s="15"/>
     </row>
-    <row r="22" spans="2:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:26" ht="18" customHeight="1">
       <c r="B22" s="246" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C22" s="247"/>
       <c r="D22" s="247"/>
@@ -5510,19 +5510,19 @@
       <c r="Y22" s="9"/>
       <c r="Z22" s="9"/>
     </row>
-    <row r="23" spans="2:26" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:26" ht="30" customHeight="1" thickBot="1">
       <c r="B23" s="160" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C23" s="255" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D23" s="233"/>
       <c r="E23" s="161" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F23" s="238" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G23" s="239"/>
       <c r="H23" s="9"/>
@@ -5545,7 +5545,7 @@
       <c r="Y23" s="9"/>
       <c r="Z23" s="9"/>
     </row>
-    <row r="24" spans="2:26" ht="9.9499999999999993" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:26" ht="9.9499999999999993" customHeight="1" thickBot="1">
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
@@ -5571,10 +5571,10 @@
       <c r="X24" s="15"/>
       <c r="Y24" s="15"/>
     </row>
-    <row r="25" spans="2:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:26" ht="18" customHeight="1" thickBot="1">
       <c r="B25" s="38"/>
       <c r="C25" s="25" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D25" s="38"/>
       <c r="E25" s="24"/>
@@ -5599,19 +5599,19 @@
       <c r="X25" s="23"/>
       <c r="Y25" s="23"/>
     </row>
-    <row r="26" spans="2:26" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:26" ht="30" customHeight="1" thickBot="1">
       <c r="B26" s="144" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C26" s="145" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D26" s="146"/>
       <c r="E26" s="147" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F26" s="145" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G26" s="145"/>
       <c r="H26" s="22"/>
@@ -5633,15 +5633,15 @@
       <c r="X26" s="23"/>
       <c r="Y26" s="23"/>
     </row>
-    <row r="27" spans="2:26" s="13" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:26" s="13" customFormat="1" ht="24.95" customHeight="1">
       <c r="B27" s="44"/>
       <c r="C27" s="81" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D27" s="82"/>
       <c r="E27" s="50"/>
       <c r="F27" s="81" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G27" s="83"/>
       <c r="H27" s="18"/>
@@ -5661,15 +5661,15 @@
       <c r="V27" s="20"/>
       <c r="Z27" s="14"/>
     </row>
-    <row r="28" spans="2:26" s="13" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:26" s="13" customFormat="1" ht="24.95" customHeight="1">
       <c r="B28" s="45"/>
       <c r="C28" s="21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D28" s="40"/>
       <c r="E28" s="51"/>
       <c r="F28" s="249" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G28" s="250"/>
       <c r="H28" s="18"/>
@@ -5689,14 +5689,14 @@
       <c r="V28" s="20"/>
       <c r="Z28" s="14"/>
     </row>
-    <row r="29" spans="2:26" s="13" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:26" s="13" customFormat="1" ht="34.5" customHeight="1">
       <c r="B29" s="46"/>
       <c r="C29" s="21" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D29" s="40"/>
       <c r="E29" s="46" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F29" s="249"/>
       <c r="G29" s="250"/>
@@ -5717,19 +5717,19 @@
       <c r="V29" s="20"/>
       <c r="Z29" s="14"/>
     </row>
-    <row r="30" spans="2:26" s="13" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:26" s="13" customFormat="1" ht="45" customHeight="1">
       <c r="B30" s="149" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C30" s="43" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D30" s="40"/>
       <c r="E30" s="52" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F30" s="21" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G30" s="40"/>
       <c r="H30" s="18"/>
@@ -5749,15 +5749,15 @@
       <c r="V30" s="20"/>
       <c r="Z30" s="14"/>
     </row>
-    <row r="31" spans="2:26" s="13" customFormat="1" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:26" s="13" customFormat="1" ht="45" customHeight="1" thickBot="1">
       <c r="B31" s="47"/>
       <c r="C31" s="21" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D31" s="41"/>
       <c r="E31" s="45"/>
       <c r="F31" s="91" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G31" s="86"/>
       <c r="H31" s="18"/>
@@ -5780,18 +5780,18 @@
       <c r="Y31" s="15"/>
       <c r="Z31" s="14"/>
     </row>
-    <row r="32" spans="2:26" s="13" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:26" s="13" customFormat="1" ht="44.25" customHeight="1">
       <c r="B32" s="47"/>
       <c r="C32" s="21" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D32" s="34"/>
       <c r="E32" s="49"/>
       <c r="F32" s="90" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G32" s="164" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H32" s="18"/>
       <c r="I32" s="18"/>
@@ -5813,17 +5813,17 @@
       <c r="Y32" s="15"/>
       <c r="Z32" s="14"/>
     </row>
-    <row r="33" spans="2:26" s="13" customFormat="1" ht="35.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:26" s="13" customFormat="1" ht="35.1" customHeight="1" thickBot="1">
       <c r="B33" s="48"/>
       <c r="C33" s="89" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D33" s="150"/>
       <c r="E33" s="87" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F33" s="42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G33" s="39"/>
       <c r="H33" s="18"/>
@@ -5846,15 +5846,15 @@
       <c r="Y33" s="15"/>
       <c r="Z33" s="14"/>
     </row>
-    <row r="34" spans="2:26" s="13" customFormat="1" ht="45.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:26" s="13" customFormat="1" ht="45.6" customHeight="1" thickBot="1">
       <c r="B34" s="49"/>
       <c r="C34" s="90" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D34" s="151"/>
       <c r="E34" s="53"/>
       <c r="F34" s="85" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G34" s="86"/>
       <c r="H34" s="18"/>
@@ -5877,19 +5877,19 @@
       <c r="Y34" s="15"/>
       <c r="Z34" s="14"/>
     </row>
-    <row r="35" spans="2:26" s="13" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:26" s="13" customFormat="1" ht="31.5" customHeight="1">
       <c r="B35" s="46" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C35" s="42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D35" s="40"/>
       <c r="E35" s="87" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F35" s="88" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G35" s="92"/>
       <c r="H35" s="18"/>
@@ -5912,15 +5912,15 @@
       <c r="Y35" s="15"/>
       <c r="Z35" s="14"/>
     </row>
-    <row r="36" spans="2:26" s="13" customFormat="1" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:26" s="13" customFormat="1" ht="46.5" customHeight="1" thickBot="1">
       <c r="B36" s="48"/>
       <c r="C36" s="84" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D36" s="86"/>
       <c r="E36" s="148"/>
       <c r="F36" s="85" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G36" s="86"/>
       <c r="H36" s="18"/>
@@ -5943,7 +5943,7 @@
       <c r="Y36" s="15"/>
       <c r="Z36" s="14"/>
     </row>
-    <row r="37" spans="2:26" s="13" customFormat="1" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:26" s="13" customFormat="1" ht="9.75" customHeight="1" thickBot="1">
       <c r="H37" s="18"/>
       <c r="I37" s="18"/>
       <c r="J37" s="19"/>
@@ -5964,24 +5964,24 @@
       <c r="Y37" s="15"/>
       <c r="Z37" s="14"/>
     </row>
-    <row r="38" spans="2:26" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:26" ht="68.25" customHeight="1">
       <c r="B38" s="93" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C38" s="94" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D38" s="95" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E38" s="95" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F38" s="95" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G38" s="96" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H38" s="18"/>
       <c r="I38" s="18"/>
@@ -6002,20 +6002,20 @@
       <c r="X38" s="18"/>
       <c r="Y38" s="18"/>
     </row>
-    <row r="39" spans="2:26" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:26" ht="52.5" customHeight="1" thickBot="1">
       <c r="B39" s="100" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C39" s="101" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D39" s="97"/>
       <c r="E39" s="97"/>
       <c r="F39" s="98" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G39" s="99" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H39" s="18"/>
       <c r="I39" s="18"/>
@@ -6036,9 +6036,9 @@
       <c r="X39" s="18"/>
       <c r="Y39" s="18"/>
     </row>
-    <row r="40" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:26" ht="15" customHeight="1">
       <c r="B40" s="256" t="s">
-        <v>203</v>
+        <v>159</v>
       </c>
       <c r="C40" s="257"/>
       <c r="D40" s="229">
@@ -6048,10 +6048,10 @@
         <v>46064</v>
       </c>
       <c r="F40" s="258" t="s">
-        <v>208</v>
+        <v>160</v>
       </c>
       <c r="G40" s="230" t="s">
-        <v>213</v>
+        <v>161</v>
       </c>
       <c r="H40" s="20"/>
       <c r="I40" s="18"/>
@@ -6072,7 +6072,7 @@
       <c r="X40" s="18"/>
       <c r="Y40" s="18"/>
     </row>
-    <row r="41" spans="2:26" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:26" ht="41.25" customHeight="1" thickBot="1">
       <c r="B41" s="225"/>
       <c r="C41" s="226"/>
       <c r="D41" s="215"/>
@@ -6098,9 +6098,9 @@
       <c r="X41" s="18"/>
       <c r="Y41" s="18"/>
     </row>
-    <row r="42" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:26" ht="15" customHeight="1">
       <c r="B42" s="221" t="s">
-        <v>204</v>
+        <v>162</v>
       </c>
       <c r="C42" s="222"/>
       <c r="D42" s="229">
@@ -6110,10 +6110,10 @@
         <v>46062</v>
       </c>
       <c r="F42" s="227" t="s">
-        <v>209</v>
+        <v>163</v>
       </c>
       <c r="G42" s="219" t="s">
-        <v>214</v>
+        <v>164</v>
       </c>
       <c r="H42" s="20"/>
       <c r="I42" s="18"/>
@@ -6134,7 +6134,7 @@
       <c r="X42" s="18"/>
       <c r="Y42" s="18"/>
     </row>
-    <row r="43" spans="2:26" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:26" ht="51.75" customHeight="1" thickBot="1">
       <c r="B43" s="225"/>
       <c r="C43" s="226"/>
       <c r="D43" s="215"/>
@@ -6160,9 +6160,9 @@
       <c r="X43" s="18"/>
       <c r="Y43" s="18"/>
     </row>
-    <row r="44" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:26">
       <c r="B44" s="221" t="s">
-        <v>205</v>
+        <v>165</v>
       </c>
       <c r="C44" s="222"/>
       <c r="D44" s="229">
@@ -6172,10 +6172,10 @@
         <v>46054</v>
       </c>
       <c r="F44" s="227" t="s">
-        <v>210</v>
+        <v>166</v>
       </c>
       <c r="G44" s="219" t="s">
-        <v>215</v>
+        <v>167</v>
       </c>
       <c r="H44" s="20"/>
       <c r="I44" s="18"/>
@@ -6196,7 +6196,7 @@
       <c r="X44" s="18"/>
       <c r="Y44" s="18"/>
     </row>
-    <row r="45" spans="2:26" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:26" ht="51.75" customHeight="1" thickBot="1">
       <c r="B45" s="225"/>
       <c r="C45" s="226"/>
       <c r="D45" s="215"/>
@@ -6222,22 +6222,22 @@
       <c r="X45" s="18"/>
       <c r="Y45" s="18"/>
     </row>
-    <row r="46" spans="2:26" ht="77.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:26" ht="77.25" customHeight="1">
       <c r="B46" s="221" t="s">
-        <v>206</v>
+        <v>168</v>
       </c>
       <c r="C46" s="222"/>
       <c r="D46" s="229">
-        <v>46054</v>
+        <v>46055</v>
       </c>
       <c r="E46" s="229">
-        <v>46054</v>
+        <v>46060</v>
       </c>
       <c r="F46" s="227" t="s">
-        <v>211</v>
+        <v>169</v>
       </c>
       <c r="G46" s="219" t="s">
-        <v>216</v>
+        <v>170</v>
       </c>
       <c r="H46" s="20"/>
       <c r="I46" s="18"/>
@@ -6258,7 +6258,7 @@
       <c r="X46" s="18"/>
       <c r="Y46" s="18"/>
     </row>
-    <row r="47" spans="2:26" ht="52.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:26" ht="52.5" hidden="1" customHeight="1">
       <c r="B47" s="225"/>
       <c r="C47" s="226"/>
       <c r="D47" s="215"/>
@@ -6284,22 +6284,22 @@
       <c r="X47" s="18"/>
       <c r="Y47" s="18"/>
     </row>
-    <row r="48" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:26" ht="15" customHeight="1">
       <c r="B48" s="221" t="s">
-        <v>207</v>
+        <v>171</v>
       </c>
       <c r="C48" s="222"/>
       <c r="D48" s="214">
-        <v>46063</v>
+        <v>46054</v>
       </c>
       <c r="E48" s="214">
-        <v>46063</v>
+        <v>46068</v>
       </c>
       <c r="F48" s="227" t="s">
-        <v>212</v>
+        <v>172</v>
       </c>
       <c r="G48" s="219" t="s">
-        <v>217</v>
+        <v>173</v>
       </c>
       <c r="H48" s="20"/>
       <c r="I48" s="18"/>
@@ -6320,7 +6320,7 @@
       <c r="X48" s="18"/>
       <c r="Y48" s="18"/>
     </row>
-    <row r="49" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:25">
       <c r="B49" s="225"/>
       <c r="C49" s="226"/>
       <c r="D49" s="215"/>
@@ -6346,7 +6346,7 @@
       <c r="X49" s="18"/>
       <c r="Y49" s="18"/>
     </row>
-    <row r="50" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:25" ht="15" customHeight="1">
       <c r="B50" s="221"/>
       <c r="C50" s="222"/>
       <c r="D50" s="214"/>
@@ -6372,7 +6372,7 @@
       <c r="X50" s="18"/>
       <c r="Y50" s="18"/>
     </row>
-    <row r="51" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:25">
       <c r="B51" s="223"/>
       <c r="C51" s="224"/>
       <c r="D51" s="216"/>
@@ -6398,7 +6398,7 @@
       <c r="X51" s="18"/>
       <c r="Y51" s="18"/>
     </row>
-    <row r="52" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:25" ht="15" customHeight="1">
       <c r="B52" s="213"/>
       <c r="C52" s="213"/>
       <c r="D52" s="214"/>
@@ -6424,7 +6424,7 @@
       <c r="X52" s="18"/>
       <c r="Y52" s="18"/>
     </row>
-    <row r="53" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:25">
       <c r="B53" s="213"/>
       <c r="C53" s="213"/>
       <c r="D53" s="216"/>
@@ -6450,7 +6450,7 @@
       <c r="X53" s="18"/>
       <c r="Y53" s="18"/>
     </row>
-    <row r="54" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:25" ht="15" customHeight="1">
       <c r="B54" s="213"/>
       <c r="C54" s="213"/>
       <c r="D54" s="214"/>
@@ -6476,7 +6476,7 @@
       <c r="X54" s="18"/>
       <c r="Y54" s="18"/>
     </row>
-    <row r="55" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:25">
       <c r="B55" s="213"/>
       <c r="C55" s="213"/>
       <c r="D55" s="216"/>
@@ -6502,7 +6502,7 @@
       <c r="X55" s="18"/>
       <c r="Y55" s="18"/>
     </row>
-    <row r="56" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:25" ht="15" customHeight="1">
       <c r="B56" s="213"/>
       <c r="C56" s="213"/>
       <c r="D56" s="214"/>
@@ -6528,7 +6528,7 @@
       <c r="X56" s="18"/>
       <c r="Y56" s="18"/>
     </row>
-    <row r="57" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:25">
       <c r="B57" s="213"/>
       <c r="C57" s="213"/>
       <c r="D57" s="215"/>
@@ -6554,7 +6554,7 @@
       <c r="X57" s="18"/>
       <c r="Y57" s="18"/>
     </row>
-    <row r="58" spans="2:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:25" ht="15" customHeight="1">
       <c r="B58" s="213"/>
       <c r="C58" s="213"/>
       <c r="D58" s="214"/>
@@ -6580,7 +6580,7 @@
       <c r="X58" s="18"/>
       <c r="Y58" s="18"/>
     </row>
-    <row r="59" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:25">
       <c r="B59" s="213"/>
       <c r="C59" s="213"/>
       <c r="D59" s="215"/>
@@ -6606,7 +6606,7 @@
       <c r="X59" s="18"/>
       <c r="Y59" s="18"/>
     </row>
-    <row r="60" spans="2:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:25" ht="15" customHeight="1" thickBot="1">
       <c r="B60" s="27"/>
       <c r="C60" s="20"/>
       <c r="D60" s="20"/>
@@ -6632,10 +6632,10 @@
       <c r="X60" s="18"/>
       <c r="Y60" s="18"/>
     </row>
-    <row r="61" spans="2:25" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:25" ht="23.25" customHeight="1">
       <c r="B61" s="102"/>
       <c r="C61" s="103" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="D61" s="104"/>
       <c r="E61" s="104"/>
@@ -6660,9 +6660,9 @@
       <c r="X61" s="22"/>
       <c r="Y61" s="22"/>
     </row>
-    <row r="62" spans="2:25" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:25" ht="19.5" customHeight="1">
       <c r="B62" s="252" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="C62" s="253"/>
       <c r="D62" s="253"/>
@@ -6688,9 +6688,9 @@
       <c r="X62" s="22"/>
       <c r="Y62" s="22"/>
     </row>
-    <row r="63" spans="2:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:25" ht="16.5" customHeight="1">
       <c r="B63" s="106" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="C63" s="28"/>
       <c r="D63" s="28"/>
@@ -6716,9 +6716,9 @@
       <c r="X63" s="29"/>
       <c r="Y63" s="29"/>
     </row>
-    <row r="64" spans="2:25" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:25" ht="16.5" customHeight="1">
       <c r="B64" s="108" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="C64" s="29"/>
       <c r="D64" s="29"/>
@@ -6744,9 +6744,9 @@
       <c r="X64" s="29"/>
       <c r="Y64" s="29"/>
     </row>
-    <row r="65" spans="2:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:26" ht="16.5" customHeight="1">
       <c r="B65" s="108" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="C65" s="29"/>
       <c r="D65" s="29"/>
@@ -6772,9 +6772,9 @@
       <c r="X65" s="29"/>
       <c r="Y65" s="29"/>
     </row>
-    <row r="66" spans="2:26" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:26" ht="16.5" customHeight="1" thickBot="1">
       <c r="B66" s="108" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="C66" s="29"/>
       <c r="D66" s="29"/>
@@ -6800,7 +6800,7 @@
       <c r="X66" s="29"/>
       <c r="Y66" s="29"/>
     </row>
-    <row r="67" spans="2:26" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:26" ht="79.5" customHeight="1">
       <c r="B67" s="115" t="s">
         <v>77</v>
       </c>
@@ -6811,13 +6811,13 @@
         <v>84</v>
       </c>
       <c r="E67" s="118" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="F67" s="117" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
       <c r="G67" s="119" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="H67" s="18"/>
       <c r="I67" s="18"/>
@@ -6839,9 +6839,9 @@
       <c r="Y67" s="18"/>
       <c r="Z67" s="18"/>
     </row>
-    <row r="68" spans="2:26" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:26" ht="32.25" customHeight="1" thickBot="1">
       <c r="B68" s="110" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="C68" s="111">
         <v>1</v>
@@ -6870,7 +6870,7 @@
       <c r="Y68" s="18"/>
       <c r="Z68" s="18"/>
     </row>
-    <row r="69" spans="2:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:26" ht="17.25" customHeight="1">
       <c r="B69" s="19"/>
       <c r="C69" s="19"/>
       <c r="D69" s="19"/>
@@ -6897,10 +6897,10 @@
       <c r="Y69" s="18"/>
       <c r="Z69" s="18"/>
     </row>
-    <row r="70" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:26" ht="15" customHeight="1">
       <c r="C70" s="30"/>
       <c r="D70" s="35" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="E70" s="30"/>
       <c r="F70" s="30"/>
@@ -6925,7 +6925,7 @@
       <c r="Y70" s="18"/>
       <c r="Z70" s="18"/>
     </row>
-    <row r="71" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:26" ht="15" customHeight="1">
       <c r="B71" s="17"/>
       <c r="C71" s="17"/>
       <c r="D71" s="17"/>
@@ -6952,7 +6952,7 @@
       <c r="Y71" s="18"/>
       <c r="Z71" s="18"/>
     </row>
-    <row r="72" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:26" ht="15" customHeight="1">
       <c r="B72" s="17"/>
       <c r="C72" s="17"/>
       <c r="D72" s="17"/>
@@ -6979,7 +6979,7 @@
       <c r="Y72" s="18"/>
       <c r="Z72" s="18"/>
     </row>
-    <row r="73" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:26" ht="15" customHeight="1" thickBot="1">
       <c r="B73" s="217"/>
       <c r="C73" s="217"/>
       <c r="D73" s="217"/>
@@ -7007,7 +7007,7 @@
       <c r="Y73" s="18"/>
       <c r="Z73" s="18"/>
     </row>
-    <row r="74" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:26" ht="15" customHeight="1">
       <c r="B74" s="251" t="s">
         <v>89</v>
       </c>
@@ -7037,7 +7037,7 @@
       <c r="Y74" s="18"/>
       <c r="Z74" s="18"/>
     </row>
-    <row r="75" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:26">
       <c r="B75" s="9"/>
       <c r="C75" s="18"/>
       <c r="D75" s="9"/>
@@ -7063,7 +7063,7 @@
       <c r="Y75" s="18"/>
       <c r="Z75" s="18"/>
     </row>
-    <row r="76" spans="2:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:26" ht="15" customHeight="1">
       <c r="B76" s="9"/>
       <c r="C76" s="18"/>
       <c r="D76" s="9"/>
@@ -7089,7 +7089,7 @@
       <c r="Y76" s="18"/>
       <c r="Z76" s="18"/>
     </row>
-    <row r="77" spans="2:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:26" ht="15" customHeight="1" thickBot="1">
       <c r="B77" s="217"/>
       <c r="C77" s="217"/>
       <c r="D77" s="217"/>
@@ -7115,14 +7115,14 @@
       <c r="Y77" s="18"/>
       <c r="Z77" s="18"/>
     </row>
-    <row r="78" spans="2:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:26" ht="15.75" customHeight="1">
       <c r="B78" s="9"/>
       <c r="C78" s="33" t="s">
         <v>93</v>
       </c>
       <c r="D78" s="9"/>
       <c r="F78" s="251" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="G78" s="251"/>
       <c r="H78" s="18"/>
@@ -7145,9 +7145,9 @@
       <c r="Y78" s="18"/>
       <c r="Z78" s="18"/>
     </row>
-    <row r="79" spans="2:26" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:26" ht="18" customHeight="1">
       <c r="B79" s="31" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="C79" s="32"/>
       <c r="D79" s="32"/>
@@ -7174,7 +7174,7 @@
       <c r="Y79" s="18"/>
       <c r="Z79" s="18"/>
     </row>
-    <row r="80" spans="2:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:26" ht="15.75" thickBot="1">
       <c r="B80" s="32"/>
       <c r="C80" s="32"/>
       <c r="D80" s="32"/>
@@ -7201,9 +7201,9 @@
       <c r="Y80" s="18"/>
       <c r="Z80" s="18"/>
     </row>
-    <row r="81" spans="2:26" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:26" ht="24" customHeight="1">
       <c r="B81" s="240" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="C81" s="241"/>
       <c r="D81" s="241"/>
@@ -7230,9 +7230,9 @@
       <c r="Y81" s="9"/>
       <c r="Z81" s="9"/>
     </row>
-    <row r="82" spans="2:26" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:26" ht="13.5" customHeight="1">
       <c r="B82" s="243" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
       <c r="C82" s="244"/>
       <c r="D82" s="244"/>
@@ -7259,7 +7259,7 @@
       <c r="Y82" s="9"/>
       <c r="Z82" s="9"/>
     </row>
-    <row r="83" spans="2:26" s="10" customFormat="1" ht="156" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:26" s="10" customFormat="1" ht="156" customHeight="1" thickBot="1">
       <c r="B83" s="121"/>
       <c r="C83" s="121"/>
       <c r="D83" s="121"/>
@@ -7267,7 +7267,7 @@
       <c r="F83" s="121"/>
       <c r="G83" s="122"/>
     </row>
-    <row r="84" spans="2:26" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:26">
       <c r="H84" s="10"/>
       <c r="I84" s="9"/>
       <c r="J84" s="9"/>
@@ -7395,64 +7395,64 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D237D29B-37DE-45D6-8EA7-98C4A952DFFE}">
   <dimension ref="D1:D12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="4:4">
       <c r="D1">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="4:4">
       <c r="D2">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="4:4">
       <c r="D3">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="4:4">
       <c r="D4">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="4:4">
       <c r="D5">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="4:4">
       <c r="D6">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="4:4">
       <c r="D7">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="4:4">
       <c r="D8">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="4:4">
       <c r="D9">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="4:4">
       <c r="D10">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="4:4">
       <c r="D11">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="4:4">
       <c r="D12">
         <v>12</v>
       </c>
@@ -7468,16 +7468,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:X24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="20" width="5.7109375" style="1" customWidth="1"/>
     <col min="21" max="24" width="8.42578125" style="1" customWidth="1"/>
     <col min="25" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" ht="18.75">
       <c r="A1" s="259" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
       <c r="B1" s="259"/>
       <c r="C1" s="259"/>
@@ -7499,13 +7499,13 @@
       <c r="S1" s="259"/>
       <c r="T1" s="259"/>
       <c r="U1" s="259" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="V1" s="259"/>
       <c r="W1" s="259"/>
       <c r="X1" s="259"/>
     </row>
-    <row r="2" spans="1:24" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" ht="33" customHeight="1">
       <c r="A2" s="259"/>
       <c r="B2" s="259"/>
       <c r="C2" s="259"/>
@@ -7527,21 +7527,21 @@
       <c r="S2" s="259"/>
       <c r="T2" s="259"/>
       <c r="U2" s="267" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="V2" s="267"/>
       <c r="W2" s="267"/>
       <c r="X2" s="267"/>
     </row>
-    <row r="3" spans="1:24" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" ht="33" customHeight="1" thickBot="1">
       <c r="U3" s="268"/>
       <c r="V3" s="268"/>
       <c r="W3" s="268"/>
       <c r="X3" s="268"/>
     </row>
-    <row r="4" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1">
       <c r="A4" s="264" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="B4" s="265"/>
       <c r="C4" s="265"/>
@@ -7556,7 +7556,7 @@
       <c r="L4" s="265"/>
       <c r="M4" s="266"/>
       <c r="N4" s="264" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="O4" s="265"/>
       <c r="P4" s="265"/>
@@ -7569,7 +7569,7 @@
       <c r="W4" s="265"/>
       <c r="X4" s="266"/>
     </row>
-    <row r="5" spans="1:24" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:24" ht="18" customHeight="1" thickBot="1">
       <c r="A5" s="261"/>
       <c r="B5" s="262"/>
       <c r="C5" s="262"/>
@@ -7595,7 +7595,7 @@
       <c r="W5" s="262"/>
       <c r="X5" s="263"/>
     </row>
-    <row r="6" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" ht="9.9499999999999993" customHeight="1">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -7621,9 +7621,9 @@
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
     </row>
-    <row r="7" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1">
       <c r="A7" s="260" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
       <c r="B7" s="260"/>
       <c r="C7" s="260"/>
@@ -7653,7 +7653,7 @@
       <c r="W7" s="260"/>
       <c r="X7" s="260"/>
     </row>
-    <row r="8" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" ht="18" customHeight="1">
       <c r="A8" s="269"/>
       <c r="B8" s="269"/>
       <c r="C8" s="269"/>
@@ -7664,7 +7664,7 @@
       <c r="H8" s="269"/>
       <c r="I8" s="269"/>
       <c r="J8" s="270" t="s">
-        <v>178</v>
+        <v>194</v>
       </c>
       <c r="K8" s="271"/>
       <c r="L8" s="271"/>
@@ -7672,7 +7672,7 @@
       <c r="N8" s="271"/>
       <c r="O8" s="272"/>
       <c r="P8" s="270" t="s">
-        <v>179</v>
+        <v>195</v>
       </c>
       <c r="Q8" s="271"/>
       <c r="R8" s="271"/>
@@ -7683,7 +7683,7 @@
       <c r="W8" s="271"/>
       <c r="X8" s="272"/>
     </row>
-    <row r="9" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" ht="9.9499999999999993" customHeight="1">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -7709,9 +7709,9 @@
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
     </row>
-    <row r="10" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" ht="18" customHeight="1">
       <c r="A10" s="273" t="s">
-        <v>180</v>
+        <v>196</v>
       </c>
       <c r="B10" s="273"/>
       <c r="C10" s="273"/>
@@ -7737,9 +7737,9 @@
       <c r="W10" s="273"/>
       <c r="X10" s="273"/>
     </row>
-    <row r="11" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" ht="18" customHeight="1">
       <c r="A11" s="274" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B11" s="274"/>
       <c r="C11" s="274"/>
@@ -7747,7 +7747,7 @@
       <c r="E11" s="274"/>
       <c r="F11" s="274"/>
       <c r="G11" s="274" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
       <c r="H11" s="274"/>
       <c r="I11" s="274"/>
@@ -7755,7 +7755,7 @@
       <c r="K11" s="274"/>
       <c r="L11" s="274"/>
       <c r="M11" s="274" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="N11" s="274"/>
       <c r="O11" s="274"/>
@@ -7763,7 +7763,7 @@
       <c r="Q11" s="274"/>
       <c r="R11" s="274"/>
       <c r="S11" s="274" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
       <c r="T11" s="274"/>
       <c r="U11" s="274"/>
@@ -7771,7 +7771,7 @@
       <c r="W11" s="274"/>
       <c r="X11" s="274"/>
     </row>
-    <row r="12" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" ht="9.9499999999999993" customHeight="1">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -7797,9 +7797,9 @@
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
     </row>
-    <row r="13" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" s="2" customFormat="1" ht="18" customHeight="1">
       <c r="A13" s="260" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="B13" s="260"/>
       <c r="C13" s="260"/>
@@ -7829,7 +7829,7 @@
       <c r="W13" s="260"/>
       <c r="X13" s="260"/>
     </row>
-    <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" ht="18" customHeight="1">
       <c r="A14" s="269"/>
       <c r="B14" s="269"/>
       <c r="C14" s="269"/>
@@ -7840,7 +7840,7 @@
       <c r="H14" s="269"/>
       <c r="I14" s="269"/>
       <c r="J14" s="270" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="K14" s="271"/>
       <c r="L14" s="271"/>
@@ -7848,7 +7848,7 @@
       <c r="N14" s="271"/>
       <c r="O14" s="272"/>
       <c r="P14" s="270" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="Q14" s="271"/>
       <c r="R14" s="271"/>
@@ -7859,7 +7859,7 @@
       <c r="W14" s="271"/>
       <c r="X14" s="272"/>
     </row>
-    <row r="15" spans="1:24" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" ht="9.9499999999999993" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -7885,9 +7885,9 @@
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
     </row>
-    <row r="16" spans="1:24" s="4" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" s="4" customFormat="1" ht="24.75" customHeight="1">
       <c r="A16" s="280" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="B16" s="280"/>
       <c r="C16" s="280"/>
@@ -7898,13 +7898,13 @@
       <c r="H16" s="280"/>
       <c r="I16" s="280"/>
       <c r="J16" s="281" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
       <c r="K16" s="281"/>
       <c r="L16" s="281"/>
       <c r="M16" s="281"/>
       <c r="N16" s="280" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="O16" s="280"/>
       <c r="P16" s="280"/>
@@ -7912,16 +7912,16 @@
       <c r="R16" s="280"/>
       <c r="S16" s="280"/>
       <c r="T16" s="282" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="U16" s="282"/>
       <c r="V16" s="282"/>
       <c r="W16" s="282"/>
       <c r="X16" s="282"/>
     </row>
-    <row r="17" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" ht="18" customHeight="1">
       <c r="A17" s="275" t="s">
-        <v>191</v>
+        <v>207</v>
       </c>
       <c r="B17" s="267"/>
       <c r="C17" s="267"/>
@@ -7932,13 +7932,13 @@
       <c r="H17" s="267"/>
       <c r="I17" s="276"/>
       <c r="J17" s="283" t="s">
-        <v>192</v>
+        <v>208</v>
       </c>
       <c r="K17" s="284"/>
       <c r="L17" s="284"/>
       <c r="M17" s="285"/>
       <c r="N17" s="275" t="s">
-        <v>193</v>
+        <v>209</v>
       </c>
       <c r="O17" s="267"/>
       <c r="P17" s="267"/>
@@ -7946,14 +7946,14 @@
       <c r="R17" s="267"/>
       <c r="S17" s="276"/>
       <c r="T17" s="275" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="U17" s="267"/>
       <c r="V17" s="267"/>
       <c r="W17" s="267"/>
       <c r="X17" s="276"/>
     </row>
-    <row r="18" spans="1:24" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" ht="48.75" customHeight="1">
       <c r="A18" s="277"/>
       <c r="B18" s="278"/>
       <c r="C18" s="278"/>
@@ -7979,11 +7979,11 @@
       <c r="W18" s="278"/>
       <c r="X18" s="279"/>
     </row>
-    <row r="19" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" ht="39" customHeight="1"/>
+    <row r="20" spans="1:24" ht="39" customHeight="1"/>
+    <row r="21" spans="1:24">
       <c r="A21" s="292" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
       <c r="B21" s="292"/>
       <c r="C21" s="292"/>
@@ -7994,7 +7994,7 @@
       <c r="H21" s="292"/>
       <c r="I21" s="5"/>
       <c r="J21" s="292" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
       <c r="K21" s="292"/>
       <c r="L21" s="292"/>
@@ -8004,7 +8004,7 @@
       <c r="P21" s="292"/>
       <c r="Q21" s="6"/>
       <c r="R21" s="292" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
       <c r="S21" s="292"/>
       <c r="T21" s="292"/>
@@ -8013,31 +8013,31 @@
       <c r="W21" s="292"/>
       <c r="X21" s="292"/>
     </row>
-    <row r="23" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:24" ht="38.25" customHeight="1">
       <c r="P23" s="289" t="s">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="Q23" s="289"/>
       <c r="R23" s="289"/>
       <c r="S23" s="289"/>
       <c r="T23" s="289"/>
       <c r="U23" s="290" t="s">
-        <v>199</v>
+        <v>215</v>
       </c>
       <c r="V23" s="290"/>
       <c r="W23" s="290"/>
       <c r="X23" s="290"/>
     </row>
-    <row r="24" spans="1:24" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" ht="38.25" customHeight="1">
       <c r="P24" s="289" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
       <c r="Q24" s="289"/>
       <c r="R24" s="289"/>
       <c r="S24" s="289"/>
       <c r="T24" s="289"/>
       <c r="U24" s="291" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="V24" s="291"/>
       <c r="W24" s="291"/>

</xml_diff>